<commit_message>
Pack: corrected 2B fixture (INV-2405 IGST, INV-2407 POS 27); Summary leads with ITC claimable now, head-wise, no netting
</commit_message>
<xml_diff>
--- a/demo/artikl_sunrise_pack.xlsx
+++ b/demo/artikl_sunrise_pack.xlsx
@@ -73,12 +73,12 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,14 +444,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -471,12 +471,16 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ITC tie-out (as per bills vs as per GSTR-2B)</t>
+          <t>ITC position by tax head (never offset one head against another)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr"/>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Bucket</t>
+        </is>
+      </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t>IGST</t>
@@ -494,260 +498,358 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Invoices</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>ITC claimable now</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>4500</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>INV-2401</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>CA to decide (in 2B, flagged; amounts as per 2B)</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>8100</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>1347</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>1347</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>INV-2403, CN-018, INV-2406, INV-2407, INV-2408, INV-2409</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Not claimable pending 2B (as per bill)</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>1395</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>1395</v>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>INV-2402, INV-2404</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>RCM: claim only after client pays the tax (as per 2B)</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>1100</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>INV-2405</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Excluded from all buckets: INV-2410, IMG-WA-991, INV-2401A (suspected duplicate / unreadable).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Head-wise tie-out: bills vs GSTR-2B (no net total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>IGST</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>CGST</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>SGST</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>ITC as per bills (extracted)</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B14" s="7" t="n">
         <v>1800</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C14" s="7" t="n">
         <v>10062</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D14" s="7" t="n">
         <v>10062</v>
       </c>
-      <c r="E6" s="5" t="n">
-        <v>21924</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>ITC as per GSTR-2B</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
-        <v>8100</v>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>6397</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>6397</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>20894</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="B15" s="7" t="n">
+        <v>9200</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>5847</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>5847</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Difference (bills − 2B)</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n">
-        <v>-6300</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>3665</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>3665</v>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>1030</v>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>Bills exclude the suspected duplicate (INV-2401A) and unreadable docs (INV-2410, IMG-WA-991). 2B includes RCM invoice INV-2405 (₹1,100 tax) — CA to confirm RCM treatment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="B16" s="7" t="n">
+        <v>-7400</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>4215</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>4215</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Pack status</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Rows fully filled</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Rows flagged (blank field + exception)</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Open HIGH exceptions (CA must clear before sign-off)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Doc</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Suggested action</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2B_UNMATCHED</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>INV-2402</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Ask client for revised 2B or drop voucher</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>GSTIN_INVALID</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>INV-2404</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Blank GSTIN; verify with client</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>RCM_SUSPECT</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>INV-2405</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Do not auto-book tax; CA decides RCM</t>
-        </is>
+          <t>Rows fully filled</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CN_VS_INV</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>CN-018</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>CA confirms credit note before books</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>POS_AMBIGUOUS</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>INV-2407</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Blank tax breakup; CA fixes POS</t>
-        </is>
+          <t>Rows flagged (blank field + exception)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>ITC_UNCLEAR</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>INV-2408</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Leave ITC flag for CA; amounts OK</t>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Open HIGH exceptions (CA must clear before sign-off)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Suggested action</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Medium: field left blank until CA decides. Low: re-upload only.</t>
+          <t>2B_UNMATCHED</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>INV-2402</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Ask client for revised 2B or drop voucher</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>GSTIN_INVALID</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>INV-2404</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Blank GSTIN; verify with client</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Checked by CA (name):</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>RCM_SUSPECT</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>INV-2405</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Do not auto-book tax; CA decides RCM</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Date:</t>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CN_VS_INV</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>CN-018</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>CA confirms credit note before books</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>POS_AMBIGUOUS</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>INV-2407</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Blank tax breakup; CA fixes POS</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>ITC_UNCLEAR</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>INV-2408</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Leave ITC flag for CA; amounts OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Medium: field left blank until CA decides. Low: re-upload only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Checked by CA (name):</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Date:</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>Prepared by Artikl (maker). Reviewed and signed by CA (checker). Artikl never files and never writes to GSTN.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A9:E9"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1649,13 +1751,13 @@
         <v>22000</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="K6" t="n">
-        <v>550</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>550</v>
+        <v>0</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>

</xml_diff>